<commit_message>
Temporary commit before rebase
</commit_message>
<xml_diff>
--- a/src/UMS_Data.xlsx
+++ b/src/UMS_Data.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="211">
   <si>
     <t>Subject Code</t>
   </si>
@@ -587,6 +587,81 @@
   </si>
   <si>
     <t>123</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Physics</t>
+  </si>
+  <si>
+    <t>wd</t>
+  </si>
+  <si>
+    <t>awd</t>
+  </si>
+  <si>
+    <t>PSCYH100</t>
+  </si>
+  <si>
+    <t>1234</t>
+  </si>
+  <si>
+    <t>FAncyNAme</t>
+  </si>
+  <si>
+    <t>FancyName</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
+    <t>1439</t>
+  </si>
+  <si>
+    <t>tom</t>
+  </si>
+  <si>
+    <t>133 westbrook</t>
+  </si>
+  <si>
+    <t>444-555</t>
+  </si>
+  <si>
+    <t>wow@gmail.com</t>
+  </si>
+  <si>
+    <t>ENG 101</t>
+  </si>
+  <si>
+    <t>wowowowow</t>
+  </si>
+  <si>
+    <t>70%</t>
+  </si>
+  <si>
+    <t>weewwooo</t>
+  </si>
+  <si>
+    <t>EV003</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>456</t>
+  </si>
+  <si>
+    <t>789</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>free</t>
+  </si>
+  <si>
+    <t>banna</t>
   </si>
 </sst>
 </file>
@@ -982,7 +1057,7 @@
     </row>
     <row r="10" spans="1:2" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>190</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>19</v>
@@ -5287,7 +5362,29 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>187</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>186</v>
+      </c>
+    </row>
     <row r="13" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="14" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="15" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -6347,7 +6444,7 @@
         <v>72</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>73</v>
+        <v>210</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>74</v>
@@ -6531,22 +6628,22 @@
     </row>
     <row r="7" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>77</v>
@@ -6555,13 +6652,13 @@
         <v>78</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>113</v>
+        <v>119</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>106</v>
       </c>
       <c r="K7" s="13">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>80</v>
@@ -6569,22 +6666,22 @@
     </row>
     <row r="8" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>77</v>
@@ -6592,14 +6689,14 @@
       <c r="H8" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I8" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>106</v>
+      <c r="I8" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>126</v>
       </c>
       <c r="K8" s="13">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>80</v>
@@ -6607,22 +6704,22 @@
     </row>
     <row r="9" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="G9" s="7" t="s">
         <v>77</v>
@@ -6630,11 +6727,11 @@
       <c r="H9" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>126</v>
+      <c r="I9" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>79</v>
       </c>
       <c r="K9" s="13">
         <v>0.5</v>
@@ -6645,22 +6742,22 @@
     </row>
     <row r="10" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>130</v>
+        <v>104</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>77</v>
@@ -6669,61 +6766,24 @@
         <v>78</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>79</v>
+        <v>14</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>137</v>
       </c>
       <c r="K10" s="13">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="K11" s="13">
-        <v>0.2</v>
-      </c>
-      <c r="L11" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
+    <row r="11" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="12" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="13" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="14" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="15" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="16" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="16" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="17" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="18" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="19" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
@@ -7707,7 +7767,44 @@
     <row r="997" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="998" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="999" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
-    <row r="1000" ht="21.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="1000">
+      <c r="A1000" t="s" s="0">
+        <v>195</v>
+      </c>
+      <c r="B1000" t="s" s="0">
+        <v>196</v>
+      </c>
+      <c r="C1000" t="s" s="0">
+        <v>197</v>
+      </c>
+      <c r="D1000" t="s" s="0">
+        <v>198</v>
+      </c>
+      <c r="E1000" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="F1000" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="G1000" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="H1000" t="s" s="0">
+        <v>186</v>
+      </c>
+      <c r="I1000" t="s" s="0">
+        <v>200</v>
+      </c>
+      <c r="J1000" t="s" s="0">
+        <v>201</v>
+      </c>
+      <c r="K1000" t="s" s="0">
+        <v>202</v>
+      </c>
+      <c r="L1000" t="s" s="0">
+        <v>203</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E5" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
@@ -8922,27 +9019,6 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="E2" s="5">
-        <v>45901.416666666664</v>
-      </c>
-      <c r="F2" s="4">
-        <v>100</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>175</v>
-      </c>
       <c r="H2" s="4" t="s">
         <v>78</v>
       </c>
@@ -8979,6 +9055,10 @@
         <v>182</v>
       </c>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
     <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="23" ht="15.75" customHeight="1" x14ac:dyDescent="0.45"/>

</xml_diff>